<commit_message>
Full RI codetype dictionaries created
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/basis.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/basis.xlsx
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes naming the unit of work an acceptance criterion is assessed over - distinct from scope, which says which features are governed. Used for the value of the basis property of diggs:AbstractAcceptanceCriterionType, inherited by both diggs:PerformanceCriterion and diggs:DesignConformanceCriterion. Where basis expresses a per-unit-length quantum, the reference length is given by the sibling baseLength element.</t>
+          <t>Codes naming the unit of work an acceptance criterion is assessed over - distinct from scope, which says which features are governed. Used for the value of the basis property of diggs:AbstractAcceptanceCriterionType, inherited by both diggs:PerformanceCriterion and diggs:DesignConformanceCriterion. Where basis expresses a per-unit-length quantum, the reference length is given by the sibling baseLength element. Extended (S14-S20 dictionary sweep) to also cover diggs:RISystemDesignType/diggs:differentialSettlementBasis, which the schema's own documentation says shares this vocabulary with AbstractAcceptanceCriterionType/basis, plus a new angular_distortion entry named in that element's documentation but previously absent from this list.</t>
         </is>
       </c>
     </row>
@@ -1202,10 +1202,31 @@
         <f>IF(ISNA(VLOOKUP(B6,AssociatedElements!B$2:B2944,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="G6" s="9" t="n"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>angular_distortion</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Angular distortion</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>The criterion or predicted value is expressed as an angular distortion (differential settlement divided by span), rather than a magnitude or a per-unit-length gradient.</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2">
@@ -1735,49 +1756,112 @@
         <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B10" s="20" t="n"/>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>per_element</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemDesign/diggs:differentialSettlementBasis</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
         <f>IF(ISNA(VLOOKUP(B11,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B11" s="20" t="n"/>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>per_unit_cell</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemDesign/diggs:differentialSettlementBasis</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
         <f>IF(ISNA(VLOOKUP(B12,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B12" s="20" t="n"/>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>per_unit_length</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemDesign/diggs:differentialSettlementBasis</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
         <f>IF(ISNA(VLOOKUP(B13,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B13" s="20" t="n"/>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>per_diameter</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemDesign/diggs:differentialSettlementBasis</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
         <f>IF(ISNA(VLOOKUP(B14,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B14" s="20" t="n"/>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>angular_distortion</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>//diggs:PerformanceCriterion/diggs:basis</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
         <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B15" s="2" t="n"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>angular_distortion</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>//diggs:DesignConformanceCriterion/diggs:basis</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
         <f>IF(ISNA(VLOOKUP(B16,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>angular_distortion</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>//diggs:RISystemDesign/diggs:differentialSettlementBasis</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17">

</xml_diff>